<commit_message>
ARI deaths to April 2026 released 29/05/2026
</commit_message>
<xml_diff>
--- a/Acute respiratory infection associated deaths, 2024-2026 (a)(b)(c)(d)(e).xlsx
+++ b/Acute respiratory infection associated deaths, 2024-2026 (a)(b)(c)(d)(e).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="33">
   <si>
     <t>Acute respiratory infection associated deaths, 2024-2026 (a)(b)(c)(d)(e)</t>
   </si>
@@ -97,7 +97,7 @@
     <t>a. Includes acute respiratory disease death registrations only. Numbers will differ to disease surveillance systems.</t>
   </si>
   <si>
-    <t>b. Includes all deaths (both doctor and coroner certified) that occurred and were registered by 31 March 2026.</t>
+    <t>b. Includes all deaths (both doctor and coroner certified) that occurred and were registered by 30 April 2026.</t>
   </si>
   <si>
     <t>c. All deaths involving COVID-19 in this report have been coded to ICD-10 codes U07.1-U07.2, U10.9 or U09.9. All deaths involving influenza have been coded to J09-J11. All deaths involving RSV have been coded to J12.1, J20.5, J21.0, B97.4.</t>
@@ -109,7 +109,7 @@
     <t>e. Refer to the methodology for more information regarding the data in this table.</t>
   </si>
   <si>
-    <t>Source: Australian Bureau of Statistics, Deaths due to acute respiratory infections in Australia March 2026</t>
+    <t>Source: Australian Bureau of Statistics, Deaths due to acute respiratory infections in Australia April 2026</t>
   </si>
 </sst>
 </file>
@@ -578,7 +578,7 @@
         <v>392</v>
       </c>
       <c r="J3" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K3" s="2">
         <v>216</v>
@@ -590,7 +590,7 @@
         <v>300</v>
       </c>
       <c r="N3" s="2">
-        <v>5120</v>
+        <v>5121</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -686,7 +686,7 @@
         <v>18</v>
       </c>
       <c r="B6" s="2">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="C6" s="2">
         <v>168</v>
@@ -701,7 +701,7 @@
         <v>152</v>
       </c>
       <c r="G6" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="H6" s="2">
         <v>360</v>
@@ -716,13 +716,13 @@
         <v>68</v>
       </c>
       <c r="L6" s="2">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="M6" s="2">
         <v>54</v>
       </c>
       <c r="N6" s="2">
-        <v>2176</v>
+        <v>2180</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -748,7 +748,7 @@
         <v>176</v>
       </c>
       <c r="H7" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="I7" s="2">
         <v>300</v>
@@ -766,7 +766,7 @@
         <v>134</v>
       </c>
       <c r="N7" s="2">
-        <v>1744</v>
+        <v>1745</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -795,7 +795,7 @@
         <v>118</v>
       </c>
       <c r="I8" s="2">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J8" s="2">
         <v>80</v>
@@ -810,7 +810,7 @@
         <v>35</v>
       </c>
       <c r="N8" s="2">
-        <v>589</v>
+        <v>590</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -821,14 +821,14 @@
         <v>72</v>
       </c>
       <c r="C9" s="2">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D9" s="2">
+        <v>58</v>
+      </c>
+      <c r="E9" s="2">
         <v>18</v>
       </c>
-      <c r="E9" t="s">
-        <v>22</v>
-      </c>
       <c r="F9" t="s">
         <v>22</v>
       </c>
@@ -854,7 +854,7 @@
         <v>22</v>
       </c>
       <c r="N9" s="2">
-        <v>135</v>
+        <v>195</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -865,13 +865,13 @@
         <v>102</v>
       </c>
       <c r="C10" s="2">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D10" s="2">
-        <v>9</v>
-      </c>
-      <c r="E10" t="s">
-        <v>22</v>
+        <v>17</v>
+      </c>
+      <c r="E10" s="2">
+        <v>5</v>
       </c>
       <c r="F10" t="s">
         <v>22</v>
@@ -898,7 +898,7 @@
         <v>22</v>
       </c>
       <c r="N10" s="2">
-        <v>138</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -909,13 +909,13 @@
         <v>24</v>
       </c>
       <c r="C11" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D11" s="2">
-        <v>17</v>
-      </c>
-      <c r="E11" t="s">
-        <v>22</v>
+        <v>30</v>
+      </c>
+      <c r="E11" s="2">
+        <v>10</v>
       </c>
       <c r="F11" t="s">
         <v>22</v>
@@ -942,7 +942,7 @@
         <v>22</v>
       </c>
       <c r="N11" s="2">
-        <v>57</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
ABS ARI deaths Released 30/07/2026
</commit_message>
<xml_diff>
--- a/Acute respiratory infection associated deaths, 2024-2026 (a)(b)(c)(d)(e).xlsx
+++ b/Acute respiratory infection associated deaths, 2024-2026 (a)(b)(c)(d)(e).xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="33">
-  <si>
-    <t>Acute respiratory infection associated deaths, 2024-2026 (a)(b)(c)(d)(e)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="26">
+  <si>
+    <t>Acute respiratory infection associated deaths, 2024-2026 (a)(b)(c)(d)</t>
   </si>
   <si>
     <t/>
@@ -88,28 +88,7 @@
     <t>2026 - RSV</t>
   </si>
   <si>
-    <t>na - not available</t>
-  </si>
-  <si>
-    <t>np - not published</t>
-  </si>
-  <si>
-    <t>a. Includes acute respiratory disease death registrations only. Numbers will differ to disease surveillance systems.</t>
-  </si>
-  <si>
-    <t>b. Includes all deaths (both doctor and coroner certified) that occurred and were registered by 30 April 2026.</t>
-  </si>
-  <si>
-    <t>c. All deaths involving COVID-19 in this report have been coded to ICD-10 codes U07.1-U07.2, U10.9 or U09.9. All deaths involving influenza have been coded to J09-J11. All deaths involving RSV have been coded to J12.1, J20.5, J21.0, B97.4.</t>
-  </si>
-  <si>
-    <t>d. Data is provisional and subject to change.</t>
-  </si>
-  <si>
-    <t>e. Refer to the methodology for more information regarding the data in this table.</t>
-  </si>
-  <si>
-    <t>Source: Australian Bureau of Statistics, Deaths due to acute respiratory infections in Australia April 2026</t>
+    <t>Source: Australian Bureau of Statistics, Deaths due to acute respiratory infections in Australia June 2026</t>
   </si>
 </sst>
 </file>
@@ -493,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -572,7 +551,7 @@
         <v>876</v>
       </c>
       <c r="H3" s="2">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="I3" s="2">
         <v>392</v>
@@ -584,13 +563,13 @@
         <v>216</v>
       </c>
       <c r="L3" s="2">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="M3" s="2">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="N3" s="2">
-        <v>5121</v>
+        <v>5126</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -657,7 +636,7 @@
         <v>68</v>
       </c>
       <c r="G5" s="2">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H5" s="2">
         <v>71</v>
@@ -678,7 +657,7 @@
         <v>19</v>
       </c>
       <c r="N5" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -686,43 +665,43 @@
         <v>18</v>
       </c>
       <c r="B6" s="2">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C6" s="2">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D6" s="2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E6" s="2">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="F6" s="2">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="G6" s="2">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="H6" s="2">
-        <v>360</v>
+        <v>370</v>
       </c>
       <c r="I6" s="2">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="J6" s="2">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="K6" s="2">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="L6" s="2">
         <v>57</v>
       </c>
       <c r="M6" s="2">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="N6" s="2">
-        <v>2180</v>
+        <v>2227</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -736,37 +715,37 @@
         <v>32</v>
       </c>
       <c r="D7" s="2">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E7" s="2">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F7" s="2">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G7" s="2">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="H7" s="2">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="I7" s="2">
-        <v>300</v>
+        <v>309</v>
       </c>
       <c r="J7" s="2">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="K7" s="2">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="L7" s="2">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M7" s="2">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="N7" s="2">
-        <v>1745</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -786,31 +765,31 @@
         <v>38</v>
       </c>
       <c r="F8" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G8" s="2">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H8" s="2">
         <v>118</v>
       </c>
       <c r="I8" s="2">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="J8" s="2">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="K8" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="L8" s="2">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M8" s="2">
         <v>35</v>
       </c>
       <c r="N8" s="2">
-        <v>590</v>
+        <v>604</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -821,19 +800,19 @@
         <v>72</v>
       </c>
       <c r="C9" s="2">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D9" s="2">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E9" s="2">
-        <v>18</v>
-      </c>
-      <c r="F9" t="s">
-        <v>22</v>
-      </c>
-      <c r="G9" t="s">
-        <v>22</v>
+        <v>61</v>
+      </c>
+      <c r="F9" s="2">
+        <v>66</v>
+      </c>
+      <c r="G9" s="2">
+        <v>24</v>
       </c>
       <c r="H9" t="s">
         <v>22</v>
@@ -854,7 +833,7 @@
         <v>22</v>
       </c>
       <c r="N9" s="2">
-        <v>195</v>
+        <v>334</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -862,22 +841,22 @@
         <v>23</v>
       </c>
       <c r="B10" s="2">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C10" s="2">
         <v>28</v>
       </c>
       <c r="D10" s="2">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E10" s="2">
-        <v>5</v>
-      </c>
-      <c r="F10" t="s">
-        <v>22</v>
-      </c>
-      <c r="G10" t="s">
-        <v>22</v>
+        <v>15</v>
+      </c>
+      <c r="F10" s="2">
+        <v>12</v>
+      </c>
+      <c r="G10" s="2">
+        <v>8</v>
       </c>
       <c r="H10" t="s">
         <v>22</v>
@@ -898,7 +877,7 @@
         <v>22</v>
       </c>
       <c r="N10" s="2">
-        <v>152</v>
+        <v>184</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -912,16 +891,16 @@
         <v>18</v>
       </c>
       <c r="D11" s="2">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E11" s="2">
-        <v>10</v>
-      </c>
-      <c r="F11" t="s">
-        <v>22</v>
-      </c>
-      <c r="G11" t="s">
-        <v>22</v>
+        <v>28</v>
+      </c>
+      <c r="F11" s="2">
+        <v>41</v>
+      </c>
+      <c r="G11" s="2">
+        <v>20</v>
       </c>
       <c r="H11" t="s">
         <v>22</v>
@@ -942,47 +921,12 @@
         <v>22</v>
       </c>
       <c r="N11" s="2">
-        <v>82</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>